<commit_message>
product upgrades round 2/3: meal planner (dropdowns, chart, live dinner panel, sheet protection, clean printing) + challenge pack expanded 4→16 verified pages at same price
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YXXCjK6mADrUUCHM2odCz1
</commit_message>
<xml_diff>
--- a/venture/07-automation/tracker/publish-queue/meal-grocery-planner-v1/Meal-Plan-Grocery-Budget-Planner.xlsx
+++ b/venture/07-automation/tracker/publish-queue/meal-grocery-planner-v1/Meal-Plan-Grocery-Budget-Planner.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="START HERE" sheetId="1" state="visible" r:id="rId3"/>
@@ -15,6 +15,17 @@
     <sheet name="Monthly Grocery Budget" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Pantry Inventory" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">'Grocery List Builder'!$B$1:$H$70</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">'Grocery List Builder'!$10:$10</definedName>
+    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">'Monthly Grocery Budget'!$B$1:$F$42</definedName>
+    <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Area" vbProcedure="false">'Pantry Inventory'!$B$1:$F$58</definedName>
+    <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Titles" vbProcedure="false">'Pantry Inventory'!$8:$8</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">'Price Book'!$B$1:$H$31</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Titles" vbProcedure="false">'Price Book'!$6:$6</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'START HERE'!$B$1:$E$39</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Weekly Meal Plan'!$B$1:$I$37</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -25,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="203">
   <si>
     <t xml:space="preserve">MEAL PLAN &amp; GROCERY BUDGET PLANNER</t>
   </si>
@@ -39,22 +50,25 @@
     <t xml:space="preserve">HOW TO USE (4 steps)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. 'Pantry Inventory' — flag Use first? = Yes on anything that should get eaten soon.</t>
+    <t xml:space="preserve">1. 'Pantry Inventory' — set Use first? to Yes (it's a dropdown) on anything that should get eaten soon.</t>
   </si>
   <si>
     <t xml:space="preserve">2. 'Weekly Meal Plan' — plan 7 days around those use-first items. Dinners first; Week 1 is a full example.</t>
   </si>
   <si>
-    <t xml:space="preserve">3. 'Grocery List Builder' — set your weekly budget in the yellow cell, list what you need with estimated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    prices, and watch 'Left vs budget'. If it goes red, swap or cut items BEFORE you're in the store.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. 'Monthly Grocery Budget' — after each week's shop, log what you really spent. The month view shows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    budget left and how the month compares to last month.</t>
+    <t xml:space="preserve">3. 'Grocery List Builder' — set your weekly budget in the yellow cell. Your chosen week's dinners appear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    on the right (pick the week number), so you build the list beside the plan. Price the items and watch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    'Left vs budget'. If it goes red, swap or cut items BEFORE you're in the store.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. 'Monthly Grocery Budget' — after each week's shop, log what you really spent. The bar chart shows each</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    week's spend against budget, and the month view compares to last month.</t>
   </si>
   <si>
     <t xml:space="preserve">THE OTHER TAB</t>
@@ -81,15 +95,27 @@
     <t xml:space="preserve">The monthly tab shows $583.17 spent of a $600 budget, $71.83 less than the month before.</t>
   </si>
   <si>
-    <t xml:space="preserve">COLOR LEGEND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yellow cells = yours to edit.  Everything else calculates automatically — please don't type over it.</t>
+    <t xml:space="preserve">COLOR LEGEND &amp; DROPDOWNS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yellow cells = yours to edit.  Everything else calculates automatically.</t>
   </si>
   <si>
     <t xml:space="preserve">Traffic lights: green = under budget (or cheapest price) · amber = right at it (or use-first) · red = over.</t>
   </si>
   <si>
+    <t xml:space="preserve">Got it?, Use first?, Where and the week picker are dropdowns — pick a value, no typing needed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each sheet is protected with NO password so formulas can't be typed over by accident. To change the</t>
+  </si>
+  <si>
+    <t xml:space="preserve">layout anyway: Review → Unprotect Sheet (Excel) — Google Sheets just shows a friendly warning instead.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every tab is print-ready: File → Print gives you one clean page-width, headers repeated.</t>
+  </si>
+  <si>
     <t xml:space="preserve">GOOGLE SHEETS USERS</t>
   </si>
   <si>
@@ -237,13 +263,19 @@
     <t xml:space="preserve">WEEK 4</t>
   </si>
   <si>
+    <t xml:space="preserve">THIS WEEK'S DINNERS</t>
+  </si>
+  <si>
     <t xml:space="preserve">GROCERY LIST BUILDER</t>
   </si>
   <si>
+    <t xml:space="preserve">Week #:</t>
+  </si>
+  <si>
     <t xml:space="preserve">Weekly grocery budget:</t>
   </si>
   <si>
-    <t xml:space="preserve">Build the list from your meal plan. If 'Left vs budget' goes red, swap or cut items BEFORE the store — that's the whole trick.</t>
+    <t xml:space="preserve">Build the list from the dinners on the right (pulled live from the Weekly Meal Plan — pick the week number). If 'Left vs budget' goes red, swap or cut items BEFORE the store.</t>
   </si>
   <si>
     <t xml:space="preserve">Grocery list total (est.):</t>
@@ -255,7 +287,7 @@
     <t xml:space="preserve">In cart so far (marked Yes):</t>
   </si>
   <si>
-    <t xml:space="preserve">Mark Got it? = Yes as you shop — 'In cart so far' keeps a running total. Type Yes exactly.</t>
+    <t xml:space="preserve">Set Got it? to Yes as you shop (it's a dropdown) — 'In cart so far' keeps a running total.</t>
   </si>
   <si>
     <t xml:space="preserve">Item</t>
@@ -534,7 +566,7 @@
     <t xml:space="preserve">Flagged use-first:</t>
   </si>
   <si>
-    <t xml:space="preserve">Shop your kitchen first. Flag Use first? = Yes on anything ageing out, then plan this week's dinners around those rows — that's food you already paid for. Type Yes exactly; the counter counts that word.</t>
+    <t xml:space="preserve">Shop your kitchen first. Set Use first? to Yes (it's a dropdown) on anything ageing out, then plan this week's dinners around those rows — that's food you already paid for.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>
@@ -619,12 +651,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\)"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="\$#,##0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -691,6 +725,19 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -774,7 +821,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -803,47 +850,63 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -851,7 +914,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -922,7 +985,7 @@
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFCCCCCC"/>
-      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF878787"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFF2CC"/>
@@ -930,7 +993,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -966,6 +1029,155 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Weekly grocery spend vs budget</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Monthly Grocery Budget'!C8</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1F3A5F"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Monthly Grocery Budget'!$B$9:$B$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Monthly Grocery Budget'!$C$9:$C$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Monthly Grocery Budget'!D8</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E7D6B"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Monthly Grocery Budget'!$B$9:$B$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Monthly Grocery Budget'!$D$9:$D$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="80"/>
+        <overlap val="-10"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="$#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>68040</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="0" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="266760" y="4381560"/>
+        <a:ext cx="5579640" cy="3239640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1146,9 +1358,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:E33"/>
+  <dimension ref="B2:E38"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1219,20 +1431,20 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="2"/>
-    </row>
-    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="3" t="s">
+      <c r="B15" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="2" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="2"/>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="3" t="s">
         <v>11</v>
       </c>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="2" t="s">
@@ -1245,20 +1457,20 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="2"/>
-    </row>
-    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="3" t="s">
+      <c r="B20" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="2" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="2" t="s">
@@ -1271,20 +1483,20 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="2"/>
-    </row>
-    <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="3" t="s">
+      <c r="B25" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="2" t="s">
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="2"/>
+    </row>
+    <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B27" s="3" t="s">
         <v>19</v>
       </c>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="2" t="s">
@@ -1292,41 +1504,67 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="2"/>
-    </row>
-    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="3" t="s">
+      <c r="B29" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="2"/>
+      <c r="B32" s="2" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="2"/>
+    </row>
+    <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="2"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="true"/>
   <mergeCells count="6">
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B8:E8"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B35:E35"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1337,7 +1575,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B2:I36"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -1349,7 +1587,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="4" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -1361,12 +1599,12 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="5" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="3" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -1378,137 +1616,137 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="7" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="7" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="7" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="7" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C12" s="6" t="n">
         <f aca="false">COUNTA(C8:I11)</f>
@@ -1517,7 +1755,7 @@
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="3" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
@@ -1529,33 +1767,33 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="7" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C16" s="8"/>
       <c r="D16" s="8"/>
@@ -1567,7 +1805,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="7" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
@@ -1579,7 +1817,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="7" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
@@ -1591,7 +1829,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="7" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C19" s="8"/>
       <c r="D19" s="8"/>
@@ -1603,7 +1841,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C20" s="6" t="n">
         <f aca="false">COUNTA(C16:I19)</f>
@@ -1612,7 +1850,7 @@
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="3" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
@@ -1624,33 +1862,33 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="7" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C24" s="8"/>
       <c r="D24" s="8"/>
@@ -1662,7 +1900,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="7" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
@@ -1674,7 +1912,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="7" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C26" s="8"/>
       <c r="D26" s="8"/>
@@ -1686,7 +1924,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="7" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C27" s="8"/>
       <c r="D27" s="8"/>
@@ -1698,7 +1936,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C28" s="6" t="n">
         <f aca="false">COUNTA(C24:I27)</f>
@@ -1707,7 +1945,7 @@
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="3" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
@@ -1719,33 +1957,33 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="6" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="7" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C32" s="8"/>
       <c r="D32" s="8"/>
@@ -1757,7 +1995,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="7" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C33" s="8"/>
       <c r="D33" s="8"/>
@@ -1769,7 +2007,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="7" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C34" s="8"/>
       <c r="D34" s="8"/>
@@ -1781,7 +2019,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="7" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C35" s="8"/>
       <c r="D35" s="8"/>
@@ -1793,7 +2031,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C36" s="6" t="n">
         <f aca="false">COUNTA(C32:I35)</f>
@@ -1801,6 +2039,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="true"/>
   <mergeCells count="5">
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="B6:I6"/>
@@ -1810,7 +2049,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1821,9 +2060,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:E70"/>
+  <dimension ref="B1:H70"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1831,611 +2070,679 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="28"/>
   </cols>
   <sheetData>
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="G1" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="H1" s="10"/>
+    </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="4" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
+      <c r="G2" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="H2" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G3" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" s="13" t="str">
+        <f aca="false">IF(INDEX('Weekly Meal Plan'!C$1:C$40,8*$H$2+2)="","",INDEX('Weekly Meal Plan'!C$1:C$40,8*$H$2+2))</f>
+        <v>Sheet-pan chicken &amp; veg</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="C4" s="10" t="n">
+        <v>78</v>
+      </c>
+      <c r="C4" s="14" t="n">
         <v>150</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" s="13" t="str">
+        <f aca="false">IF(INDEX('Weekly Meal Plan'!D$1:D$40,8*$H$2+2)="","",INDEX('Weekly Meal Plan'!D$1:D$40,8*$H$2+2))</f>
+        <v>Big-batch chili</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="5" t="s">
-        <v>72</v>
+        <v>79</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H5" s="13" t="str">
+        <f aca="false">IF(INDEX('Weekly Meal Plan'!E$1:E$40,8*$H$2+2)="","",INDEX('Weekly Meal Plan'!E$1:E$40,8*$H$2+2))</f>
+        <v>Taco night</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="C6" s="11" t="n">
+        <v>80</v>
+      </c>
+      <c r="C6" s="15" t="n">
         <f aca="false">C20+C30+C40+C50+C60+C70</f>
         <v>134.86</v>
       </c>
+      <c r="G6" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="13" t="str">
+        <f aca="false">IF(INDEX('Weekly Meal Plan'!F$1:F$40,8*$H$2+2)="","",INDEX('Weekly Meal Plan'!F$1:F$40,8*$H$2+2))</f>
+        <v>Pasta marinara</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="C7" s="12" t="n">
+        <v>81</v>
+      </c>
+      <c r="C7" s="16" t="n">
         <f aca="false">C4-C6</f>
         <v>15.14</v>
       </c>
+      <c r="G7" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="H7" s="13" t="str">
+        <f aca="false">IF(INDEX('Weekly Meal Plan'!G$1:G$40,8*$H$2+2)="","",INDEX('Weekly Meal Plan'!G$1:G$40,8*$H$2+2))</f>
+        <v>Chicken stir-fry</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="C8" s="11" t="n">
+        <v>82</v>
+      </c>
+      <c r="C8" s="15" t="n">
         <f aca="false">SUMIF(D12:D69,"Yes",C12:C69)</f>
         <v>22.92</v>
       </c>
+      <c r="G8" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H8" s="13" t="str">
+        <f aca="false">IF(INDEX('Weekly Meal Plan'!H$1:H$40,8*$H$2+2)="","",INDEX('Weekly Meal Plan'!H$1:H$40,8*$H$2+2))</f>
+        <v>Homemade pizza</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="5" t="s">
-        <v>76</v>
+        <v>83</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H9" s="13" t="str">
+        <f aca="false">IF(INDEX('Weekly Meal Plan'!I$1:I$40,8*$H$2+2)="","",INDEX('Weekly Meal Plan'!I$1:I$40,8*$H$2+2))</f>
+        <v>Leftovers night</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="C12" s="10" t="n">
+      <c r="B12" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" s="14" t="n">
         <v>2.28</v>
       </c>
-      <c r="D12" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="E12" s="13"/>
+      <c r="D12" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="E12" s="17"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="C13" s="10" t="n">
+      <c r="B13" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="C13" s="14" t="n">
         <v>4.49</v>
       </c>
-      <c r="D13" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="E13" s="13"/>
+      <c r="D13" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="E13" s="17"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="C14" s="10" t="n">
+      <c r="B14" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C14" s="14" t="n">
         <v>2.29</v>
       </c>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="C15" s="10" t="n">
+      <c r="B15" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="C15" s="14" t="n">
         <v>3.99</v>
       </c>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="C16" s="10" t="n">
+      <c r="B16" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="C16" s="14" t="n">
         <v>3.49</v>
       </c>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="C17" s="10" t="n">
+      <c r="B17" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="C17" s="14" t="n">
         <v>2.79</v>
       </c>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="C18" s="10" t="n">
+      <c r="B18" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="C18" s="14" t="n">
         <v>2.99</v>
       </c>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="C19" s="10" t="n">
+      <c r="B19" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="C19" s="14" t="n">
         <v>2.99</v>
       </c>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="C20" s="11" t="n">
+        <v>97</v>
+      </c>
+      <c r="C20" s="15" t="n">
         <f aca="false">SUM(C12:C19)</f>
         <v>25.31</v>
       </c>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C22" s="10" t="n">
+      <c r="B22" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="C22" s="14" t="n">
         <v>8.97</v>
       </c>
-      <c r="D22" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="E22" s="13"/>
+      <c r="D22" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="E22" s="17"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="C23" s="10" t="n">
+      <c r="B23" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="C23" s="14" t="n">
         <v>9.98</v>
       </c>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="C24" s="10" t="n">
+      <c r="B24" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="C24" s="14" t="n">
         <v>4.99</v>
       </c>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="C25" s="10" t="n">
+      <c r="B25" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="C25" s="14" t="n">
         <v>4.36</v>
       </c>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="13"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="13"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="13"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="13"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C30" s="11" t="n">
+        <v>103</v>
+      </c>
+      <c r="C30" s="15" t="n">
         <f aca="false">SUM(C22:C29)</f>
         <v>28.3</v>
       </c>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
     </row>
     <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="3" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="C32" s="10" t="n">
+      <c r="B32" s="17" t="s">
+        <v>105</v>
+      </c>
+      <c r="C32" s="14" t="n">
         <v>7.18</v>
       </c>
-      <c r="D32" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="E32" s="13"/>
+      <c r="D32" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="E32" s="17"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="C33" s="10" t="n">
+      <c r="B33" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="C33" s="14" t="n">
         <v>4.79</v>
       </c>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="C34" s="10" t="n">
+      <c r="B34" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="C34" s="14" t="n">
         <v>5.49</v>
       </c>
-      <c r="D34" s="13"/>
-      <c r="E34" s="13"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="C35" s="10" t="n">
+      <c r="B35" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="C35" s="14" t="n">
         <v>3.79</v>
       </c>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="C36" s="10" t="n">
+      <c r="B36" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="C36" s="14" t="n">
         <v>3.99</v>
       </c>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="13"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="13"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
+      <c r="B38" s="17"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="13"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13"/>
+      <c r="B39" s="17"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="17"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="C40" s="11" t="n">
+        <v>110</v>
+      </c>
+      <c r="C40" s="15" t="n">
         <f aca="false">SUM(C32:C39)</f>
         <v>25.24</v>
       </c>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="18"/>
     </row>
     <row r="41" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="3" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="13" t="s">
-        <v>105</v>
-      </c>
-      <c r="C42" s="10" t="n">
+      <c r="B42" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="C42" s="14" t="n">
         <v>4.29</v>
       </c>
-      <c r="D42" s="13"/>
-      <c r="E42" s="13"/>
+      <c r="D42" s="17"/>
+      <c r="E42" s="17"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="C43" s="10" t="n">
+      <c r="B43" s="17" t="s">
+        <v>113</v>
+      </c>
+      <c r="C43" s="14" t="n">
         <v>2.58</v>
       </c>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
+      <c r="D43" s="17"/>
+      <c r="E43" s="17"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="C44" s="10" t="n">
+      <c r="B44" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="C44" s="14" t="n">
         <v>4.58</v>
       </c>
-      <c r="D44" s="13"/>
-      <c r="E44" s="13"/>
+      <c r="D44" s="17"/>
+      <c r="E44" s="17"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="C45" s="10" t="n">
+      <c r="B45" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="C45" s="14" t="n">
         <v>5.49</v>
       </c>
-      <c r="D45" s="13"/>
-      <c r="E45" s="13"/>
+      <c r="D45" s="17"/>
+      <c r="E45" s="17"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="C46" s="10" t="n">
+      <c r="B46" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="C46" s="14" t="n">
         <v>3.79</v>
       </c>
-      <c r="D46" s="13"/>
-      <c r="E46" s="13"/>
+      <c r="D46" s="17"/>
+      <c r="E46" s="17"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="C47" s="10" t="n">
+      <c r="B47" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="C47" s="14" t="n">
         <v>5.18</v>
       </c>
-      <c r="D47" s="13"/>
-      <c r="E47" s="13"/>
+      <c r="D47" s="17"/>
+      <c r="E47" s="17"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="C48" s="10" t="n">
+      <c r="B48" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="C48" s="14" t="n">
         <v>3.29</v>
       </c>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13"/>
+      <c r="D48" s="17"/>
+      <c r="E48" s="17"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="C49" s="10" t="n">
+      <c r="B49" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="C49" s="14" t="n">
         <v>0.99</v>
       </c>
-      <c r="D49" s="13"/>
-      <c r="E49" s="13"/>
+      <c r="D49" s="17"/>
+      <c r="E49" s="17"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="C50" s="11" t="n">
+        <v>120</v>
+      </c>
+      <c r="C50" s="15" t="n">
         <f aca="false">SUM(C42:C49)</f>
         <v>30.19</v>
       </c>
-      <c r="D50" s="14"/>
-      <c r="E50" s="14"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="18"/>
     </row>
     <row r="51" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="3" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="C52" s="10" t="n">
+      <c r="B52" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="C52" s="14" t="n">
         <v>3.87</v>
       </c>
-      <c r="D52" s="13"/>
-      <c r="E52" s="13"/>
+      <c r="D52" s="17"/>
+      <c r="E52" s="17"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="C53" s="10" t="n">
+      <c r="B53" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="C53" s="14" t="n">
         <v>3.99</v>
       </c>
-      <c r="D53" s="13"/>
-      <c r="E53" s="13"/>
+      <c r="D53" s="17"/>
+      <c r="E53" s="17"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="C54" s="10" t="n">
+      <c r="B54" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="C54" s="14" t="n">
         <v>2.49</v>
       </c>
-      <c r="D54" s="13"/>
-      <c r="E54" s="13"/>
+      <c r="D54" s="17"/>
+      <c r="E54" s="17"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="13"/>
-      <c r="C55" s="10"/>
-      <c r="D55" s="13"/>
-      <c r="E55" s="13"/>
+      <c r="B55" s="17"/>
+      <c r="C55" s="14"/>
+      <c r="D55" s="17"/>
+      <c r="E55" s="17"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="13"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="13"/>
-      <c r="E56" s="13"/>
+      <c r="B56" s="17"/>
+      <c r="C56" s="14"/>
+      <c r="D56" s="17"/>
+      <c r="E56" s="17"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="13"/>
-      <c r="C57" s="10"/>
-      <c r="D57" s="13"/>
-      <c r="E57" s="13"/>
+      <c r="B57" s="17"/>
+      <c r="C57" s="14"/>
+      <c r="D57" s="17"/>
+      <c r="E57" s="17"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="13"/>
-      <c r="C58" s="10"/>
-      <c r="D58" s="13"/>
-      <c r="E58" s="13"/>
+      <c r="B58" s="17"/>
+      <c r="C58" s="14"/>
+      <c r="D58" s="17"/>
+      <c r="E58" s="17"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="13"/>
-      <c r="C59" s="10"/>
-      <c r="D59" s="13"/>
-      <c r="E59" s="13"/>
+      <c r="B59" s="17"/>
+      <c r="C59" s="14"/>
+      <c r="D59" s="17"/>
+      <c r="E59" s="17"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="C60" s="11" t="n">
+        <v>125</v>
+      </c>
+      <c r="C60" s="15" t="n">
         <f aca="false">SUM(C52:C59)</f>
         <v>10.35</v>
       </c>
-      <c r="D60" s="14"/>
-      <c r="E60" s="14"/>
+      <c r="D60" s="18"/>
+      <c r="E60" s="18"/>
     </row>
     <row r="61" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B61" s="3" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
       <c r="E61" s="3"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B62" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="C62" s="10" t="n">
+      <c r="B62" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="C62" s="14" t="n">
         <v>2.99</v>
       </c>
-      <c r="D62" s="13"/>
-      <c r="E62" s="13"/>
+      <c r="D62" s="17"/>
+      <c r="E62" s="17"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="C63" s="10" t="n">
+      <c r="B63" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="C63" s="14" t="n">
         <v>5.99</v>
       </c>
-      <c r="D63" s="13"/>
-      <c r="E63" s="13"/>
+      <c r="D63" s="17"/>
+      <c r="E63" s="17"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B64" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="C64" s="10" t="n">
+      <c r="B64" s="17" t="s">
+        <v>129</v>
+      </c>
+      <c r="C64" s="14" t="n">
         <v>6.49</v>
       </c>
-      <c r="D64" s="13"/>
-      <c r="E64" s="13"/>
+      <c r="D64" s="17"/>
+      <c r="E64" s="17"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B65" s="13"/>
-      <c r="C65" s="10"/>
-      <c r="D65" s="13"/>
-      <c r="E65" s="13"/>
+      <c r="B65" s="17"/>
+      <c r="C65" s="14"/>
+      <c r="D65" s="17"/>
+      <c r="E65" s="17"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B66" s="13"/>
-      <c r="C66" s="10"/>
-      <c r="D66" s="13"/>
-      <c r="E66" s="13"/>
+      <c r="B66" s="17"/>
+      <c r="C66" s="14"/>
+      <c r="D66" s="17"/>
+      <c r="E66" s="17"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B67" s="13"/>
-      <c r="C67" s="10"/>
-      <c r="D67" s="13"/>
-      <c r="E67" s="13"/>
+      <c r="B67" s="17"/>
+      <c r="C67" s="14"/>
+      <c r="D67" s="17"/>
+      <c r="E67" s="17"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B68" s="13"/>
-      <c r="C68" s="10"/>
-      <c r="D68" s="13"/>
-      <c r="E68" s="13"/>
+      <c r="B68" s="17"/>
+      <c r="C68" s="14"/>
+      <c r="D68" s="17"/>
+      <c r="E68" s="17"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B69" s="13"/>
-      <c r="C69" s="10"/>
-      <c r="D69" s="13"/>
-      <c r="E69" s="13"/>
+      <c r="B69" s="17"/>
+      <c r="C69" s="14"/>
+      <c r="D69" s="17"/>
+      <c r="E69" s="17"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="C70" s="11" t="n">
+        <v>130</v>
+      </c>
+      <c r="C70" s="15" t="n">
         <f aca="false">SUM(C62:C69)</f>
         <v>15.47</v>
       </c>
-      <c r="D70" s="14"/>
-      <c r="E70" s="14"/>
+      <c r="D70" s="18"/>
+      <c r="E70" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <sheetProtection sheet="true"/>
+  <mergeCells count="8">
+    <mergeCell ref="G1:H1"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B11:E11"/>
     <mergeCell ref="B21:E21"/>
@@ -2455,9 +2762,19 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" error="Pick a week number from 1 to 4." errorStyle="stop" errorTitle="Pick from the dropdown" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2" type="list">
+      <formula1>"1,2,3,4"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Pick Yes (in the cart) or No — the running total counts Yes." errorStyle="stop" errorTitle="Pick from the dropdown" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D12:D19 D22:D29 D32:D39 D42:D49 D52:D59 D62:D69" type="list">
+      <formula1>"Yes,No"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -2468,7 +2785,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B2:H31"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -2483,7 +2800,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="4" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -2494,513 +2811,514 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="5" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="5" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>130</v>
+        <v>134</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>137</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="D7" s="10" t="n">
+      <c r="B7" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="D7" s="14" t="n">
         <v>3.89</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="14" t="n">
         <v>3.59</v>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="14" t="n">
         <v>3.29</v>
       </c>
-      <c r="G7" s="16" t="str">
+      <c r="G7" s="20" t="str">
         <f aca="false">IF(COUNT(D7:F7)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D7:F7),D7:F7,0)))</f>
         <v>Store 3</v>
       </c>
-      <c r="H7" s="17" t="n">
+      <c r="H7" s="21" t="n">
         <f aca="false">IF(COUNT(D7:F7)=0,"",MIN(D7:F7))</f>
         <v>3.29</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>135</v>
-      </c>
-      <c r="D8" s="10" t="n">
+      <c r="B8" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="D8" s="14" t="n">
         <v>4.97</v>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" s="14" t="n">
         <v>5.29</v>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="F8" s="14" t="n">
         <v>4.39</v>
       </c>
-      <c r="G8" s="16" t="str">
+      <c r="G8" s="20" t="str">
         <f aca="false">IF(COUNT(D8:F8)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D8:F8),D8:F8,0)))</f>
         <v>Store 3</v>
       </c>
-      <c r="H8" s="17" t="n">
+      <c r="H8" s="21" t="n">
         <f aca="false">IF(COUNT(D8:F8)=0,"",MIN(D8:F8))</f>
         <v>4.39</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>137</v>
-      </c>
-      <c r="D9" s="10" t="n">
+      <c r="B9" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="D9" s="14" t="n">
         <v>3.49</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="14" t="n">
         <v>2.99</v>
       </c>
-      <c r="F9" s="10" t="n">
+      <c r="F9" s="14" t="n">
         <v>3.19</v>
       </c>
-      <c r="G9" s="16" t="str">
+      <c r="G9" s="20" t="str">
         <f aca="false">IF(COUNT(D9:F9)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D9:F9),D9:F9,0)))</f>
         <v>Store 2</v>
       </c>
-      <c r="H9" s="17" t="n">
+      <c r="H9" s="21" t="n">
         <f aca="false">IF(COUNT(D9:F9)=0,"",MIN(D9:F9))</f>
         <v>2.99</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>137</v>
-      </c>
-      <c r="D10" s="10" t="n">
+      <c r="B10" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="D10" s="14" t="n">
         <v>4.87</v>
       </c>
-      <c r="E10" s="10" t="n">
+      <c r="E10" s="14" t="n">
         <v>4.99</v>
       </c>
-      <c r="F10" s="10" t="n">
+      <c r="F10" s="14" t="n">
         <v>4.49</v>
       </c>
-      <c r="G10" s="16" t="str">
+      <c r="G10" s="20" t="str">
         <f aca="false">IF(COUNT(D10:F10)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D10:F10),D10:F10,0)))</f>
         <v>Store 3</v>
       </c>
-      <c r="H10" s="17" t="n">
+      <c r="H10" s="21" t="n">
         <f aca="false">IF(COUNT(D10:F10)=0,"",MIN(D10:F10))</f>
         <v>4.49</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="13" t="s">
-        <v>139</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>140</v>
-      </c>
-      <c r="D11" s="10" t="n">
+      <c r="B11" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="D11" s="14" t="n">
         <v>2.59</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="14" t="n">
         <v>2.49</v>
       </c>
-      <c r="F11" s="10" t="n">
+      <c r="F11" s="14" t="n">
         <v>1.99</v>
       </c>
-      <c r="G11" s="16" t="str">
+      <c r="G11" s="20" t="str">
         <f aca="false">IF(COUNT(D11:F11)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D11:F11),D11:F11,0)))</f>
         <v>Store 3</v>
       </c>
-      <c r="H11" s="17" t="n">
+      <c r="H11" s="21" t="n">
         <f aca="false">IF(COUNT(D11:F11)=0,"",MIN(D11:F11))</f>
         <v>1.99</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>137</v>
-      </c>
-      <c r="D12" s="10" t="n">
+      <c r="B12" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="D12" s="14" t="n">
         <v>0.54</v>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E12" s="14" t="n">
         <v>0.59</v>
       </c>
-      <c r="F12" s="10" t="n">
+      <c r="F12" s="14" t="n">
         <v>0.44</v>
       </c>
-      <c r="G12" s="16" t="str">
+      <c r="G12" s="20" t="str">
         <f aca="false">IF(COUNT(D12:F12)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D12:F12),D12:F12,0)))</f>
         <v>Store 3</v>
       </c>
-      <c r="H12" s="17" t="n">
+      <c r="H12" s="21" t="n">
         <f aca="false">IF(COUNT(D12:F12)=0,"",MIN(D12:F12))</f>
         <v>0.44</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="D13" s="10" t="n">
+      <c r="B13" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="D13" s="14" t="n">
         <v>2.48</v>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="14" t="n">
         <v>3.29</v>
       </c>
-      <c r="F13" s="10" t="n">
+      <c r="F13" s="14" t="n">
         <v>2.79</v>
       </c>
-      <c r="G13" s="16" t="str">
+      <c r="G13" s="20" t="str">
         <f aca="false">IF(COUNT(D13:F13)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D13:F13),D13:F13,0)))</f>
         <v>Store 1</v>
       </c>
-      <c r="H13" s="17" t="n">
+      <c r="H13" s="21" t="n">
         <f aca="false">IF(COUNT(D13:F13)=0,"",MIN(D13:F13))</f>
         <v>2.48</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="D14" s="10" t="n">
+      <c r="B14" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="D14" s="14" t="n">
         <v>1.24</v>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E14" s="14" t="n">
         <v>0.99</v>
       </c>
-      <c r="F14" s="10" t="n">
+      <c r="F14" s="14" t="n">
         <v>1.09</v>
       </c>
-      <c r="G14" s="16" t="str">
+      <c r="G14" s="20" t="str">
         <f aca="false">IF(COUNT(D14:F14)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D14:F14),D14:F14,0)))</f>
         <v>Store 2</v>
       </c>
-      <c r="H14" s="17" t="n">
+      <c r="H14" s="21" t="n">
         <f aca="false">IF(COUNT(D14:F14)=0,"",MIN(D14:F14))</f>
         <v>0.99</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="D15" s="10" t="n">
+      <c r="B15" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>151</v>
+      </c>
+      <c r="D15" s="14" t="n">
         <v>4.97</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E15" s="14" t="n">
         <v>5.49</v>
       </c>
-      <c r="F15" s="10" t="n">
+      <c r="F15" s="14" t="n">
         <v>5.29</v>
       </c>
-      <c r="G15" s="16" t="str">
+      <c r="G15" s="20" t="str">
         <f aca="false">IF(COUNT(D15:F15)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D15:F15),D15:F15,0)))</f>
         <v>Store 1</v>
       </c>
-      <c r="H15" s="17" t="n">
+      <c r="H15" s="21" t="n">
         <f aca="false">IF(COUNT(D15:F15)=0,"",MIN(D15:F15))</f>
         <v>4.97</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D16" s="10" t="n">
+      <c r="B16" s="17" t="s">
+        <v>152</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="D16" s="14" t="n">
         <v>2.87</v>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E16" s="14" t="n">
         <v>2.5</v>
       </c>
-      <c r="F16" s="10" t="n">
+      <c r="F16" s="14" t="n">
         <v>2.29</v>
       </c>
-      <c r="G16" s="16" t="str">
+      <c r="G16" s="20" t="str">
         <f aca="false">IF(COUNT(D16:F16)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D16:F16),D16:F16,0)))</f>
         <v>Store 3</v>
       </c>
-      <c r="H16" s="17" t="n">
+      <c r="H16" s="21" t="n">
         <f aca="false">IF(COUNT(D16:F16)=0,"",MIN(D16:F16))</f>
         <v>2.29</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="16" t="str">
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="20" t="str">
         <f aca="false">IF(COUNT(D17:F17)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D17:F17),D17:F17,0)))</f>
         <v/>
       </c>
-      <c r="H17" s="17" t="str">
+      <c r="H17" s="21" t="str">
         <f aca="false">IF(COUNT(D17:F17)=0,"",MIN(D17:F17))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="16" t="str">
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="20" t="str">
         <f aca="false">IF(COUNT(D18:F18)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D18:F18),D18:F18,0)))</f>
         <v/>
       </c>
-      <c r="H18" s="17" t="str">
+      <c r="H18" s="21" t="str">
         <f aca="false">IF(COUNT(D18:F18)=0,"",MIN(D18:F18))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="16" t="str">
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="20" t="str">
         <f aca="false">IF(COUNT(D19:F19)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D19:F19),D19:F19,0)))</f>
         <v/>
       </c>
-      <c r="H19" s="17" t="str">
+      <c r="H19" s="21" t="str">
         <f aca="false">IF(COUNT(D19:F19)=0,"",MIN(D19:F19))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="16" t="str">
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="20" t="str">
         <f aca="false">IF(COUNT(D20:F20)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D20:F20),D20:F20,0)))</f>
         <v/>
       </c>
-      <c r="H20" s="17" t="str">
+      <c r="H20" s="21" t="str">
         <f aca="false">IF(COUNT(D20:F20)=0,"",MIN(D20:F20))</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="16" t="str">
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="20" t="str">
         <f aca="false">IF(COUNT(D21:F21)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D21:F21),D21:F21,0)))</f>
         <v/>
       </c>
-      <c r="H21" s="17" t="str">
+      <c r="H21" s="21" t="str">
         <f aca="false">IF(COUNT(D21:F21)=0,"",MIN(D21:F21))</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="16" t="str">
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="20" t="str">
         <f aca="false">IF(COUNT(D22:F22)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D22:F22),D22:F22,0)))</f>
         <v/>
       </c>
-      <c r="H22" s="17" t="str">
+      <c r="H22" s="21" t="str">
         <f aca="false">IF(COUNT(D22:F22)=0,"",MIN(D22:F22))</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="16" t="str">
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="20" t="str">
         <f aca="false">IF(COUNT(D23:F23)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D23:F23),D23:F23,0)))</f>
         <v/>
       </c>
-      <c r="H23" s="17" t="str">
+      <c r="H23" s="21" t="str">
         <f aca="false">IF(COUNT(D23:F23)=0,"",MIN(D23:F23))</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="16" t="str">
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="20" t="str">
         <f aca="false">IF(COUNT(D24:F24)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D24:F24),D24:F24,0)))</f>
         <v/>
       </c>
-      <c r="H24" s="17" t="str">
+      <c r="H24" s="21" t="str">
         <f aca="false">IF(COUNT(D24:F24)=0,"",MIN(D24:F24))</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="16" t="str">
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="20" t="str">
         <f aca="false">IF(COUNT(D25:F25)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D25:F25),D25:F25,0)))</f>
         <v/>
       </c>
-      <c r="H25" s="17" t="str">
+      <c r="H25" s="21" t="str">
         <f aca="false">IF(COUNT(D25:F25)=0,"",MIN(D25:F25))</f>
         <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="16" t="str">
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="20" t="str">
         <f aca="false">IF(COUNT(D26:F26)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D26:F26),D26:F26,0)))</f>
         <v/>
       </c>
-      <c r="H26" s="17" t="str">
+      <c r="H26" s="21" t="str">
         <f aca="false">IF(COUNT(D26:F26)=0,"",MIN(D26:F26))</f>
         <v/>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="16" t="str">
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="20" t="str">
         <f aca="false">IF(COUNT(D27:F27)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D27:F27),D27:F27,0)))</f>
         <v/>
       </c>
-      <c r="H27" s="17" t="str">
+      <c r="H27" s="21" t="str">
         <f aca="false">IF(COUNT(D27:F27)=0,"",MIN(D27:F27))</f>
         <v/>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="16" t="str">
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="20" t="str">
         <f aca="false">IF(COUNT(D28:F28)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D28:F28),D28:F28,0)))</f>
         <v/>
       </c>
-      <c r="H28" s="17" t="str">
+      <c r="H28" s="21" t="str">
         <f aca="false">IF(COUNT(D28:F28)=0,"",MIN(D28:F28))</f>
         <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="13"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="16" t="str">
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="20" t="str">
         <f aca="false">IF(COUNT(D29:F29)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D29:F29),D29:F29,0)))</f>
         <v/>
       </c>
-      <c r="H29" s="17" t="str">
+      <c r="H29" s="21" t="str">
         <f aca="false">IF(COUNT(D29:F29)=0,"",MIN(D29:F29))</f>
         <v/>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
-      <c r="G30" s="16" t="str">
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="20" t="str">
         <f aca="false">IF(COUNT(D30:F30)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D30:F30),D30:F30,0)))</f>
         <v/>
       </c>
-      <c r="H30" s="17" t="str">
+      <c r="H30" s="21" t="str">
         <f aca="false">IF(COUNT(D30:F30)=0,"",MIN(D30:F30))</f>
         <v/>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="16" t="str">
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="20" t="str">
         <f aca="false">IF(COUNT(D31:F31)=0,"",INDEX($D$6:$F$6,MATCH(MIN(D31:F31),D31:F31,0)))</f>
         <v/>
       </c>
-      <c r="H31" s="17" t="str">
+      <c r="H31" s="21" t="str">
         <f aca="false">IF(COUNT(D31:F31)=0,"",MIN(D31:F31))</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="true"/>
   <mergeCells count="1">
     <mergeCell ref="B2:H2"/>
   </mergeCells>
@@ -3011,7 +3329,7 @@
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3022,7 +3340,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B2:E21"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -3034,7 +3352,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="4" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -3042,170 +3360,171 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="C4" s="10" t="n">
+        <v>155</v>
+      </c>
+      <c r="C4" s="14" t="n">
         <v>600</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="C5" s="10" t="n">
+        <v>156</v>
+      </c>
+      <c r="C5" s="14" t="n">
         <v>655</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="5" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="16" t="s">
-        <v>155</v>
-      </c>
-      <c r="C9" s="17" t="n">
+      <c r="B9" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="C9" s="21" t="n">
         <f aca="false">$C$4/4</f>
         <v>150</v>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="14" t="n">
         <v>138.42</v>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="E9" s="21" t="n">
         <f aca="false">C9-D9</f>
         <v>11.58</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="16" t="s">
-        <v>156</v>
-      </c>
-      <c r="C10" s="17" t="n">
+      <c r="B10" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="C10" s="21" t="n">
         <f aca="false">$C$4/4</f>
         <v>150</v>
       </c>
-      <c r="D10" s="10" t="n">
+      <c r="D10" s="14" t="n">
         <v>161.85</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="E10" s="21" t="n">
         <f aca="false">C10-D10</f>
         <v>-11.85</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="16" t="s">
-        <v>157</v>
-      </c>
-      <c r="C11" s="17" t="n">
+      <c r="B11" s="20" t="s">
+        <v>164</v>
+      </c>
+      <c r="C11" s="21" t="n">
         <f aca="false">$C$4/4</f>
         <v>150</v>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="D11" s="14" t="n">
         <v>150</v>
       </c>
-      <c r="E11" s="17" t="n">
+      <c r="E11" s="21" t="n">
         <f aca="false">C11-D11</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="C12" s="17" t="n">
+      <c r="B12" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="C12" s="21" t="n">
         <f aca="false">$C$4/4</f>
         <v>150</v>
       </c>
-      <c r="D12" s="10" t="n">
+      <c r="D12" s="14" t="n">
         <v>132.9</v>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="E12" s="21" t="n">
         <f aca="false">C12-D12</f>
         <v>17.1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="C13" s="11" t="n">
+        <v>166</v>
+      </c>
+      <c r="C13" s="15" t="n">
         <f aca="false">SUM(C9:C12)</f>
         <v>600</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="15" t="n">
         <f aca="false">SUM(D9:D12)</f>
         <v>583.17</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="15" t="n">
         <f aca="false">C13-D13</f>
         <v>16.83</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="18" t="s">
-        <v>160</v>
-      </c>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
+      <c r="B15" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="C16" s="12" t="n">
+        <v>168</v>
+      </c>
+      <c r="C16" s="16" t="n">
         <f aca="false">D13</f>
         <v>583.17</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="9" t="s">
-        <v>162</v>
-      </c>
-      <c r="C17" s="12" t="n">
+        <v>169</v>
+      </c>
+      <c r="C17" s="16" t="n">
         <f aca="false">C4-D13</f>
         <v>16.83</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="9" t="s">
-        <v>163</v>
-      </c>
-      <c r="C18" s="19" t="n">
+        <v>170</v>
+      </c>
+      <c r="C18" s="23" t="n">
         <f aca="false">IF(C4=0,"",D13/C4)</f>
         <v>0.97195</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="C19" s="12" t="n">
+        <v>171</v>
+      </c>
+      <c r="C19" s="16" t="n">
         <f aca="false">C5-D13</f>
         <v>71.83</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="5" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="true"/>
   <mergeCells count="2">
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B15:E15"/>
@@ -3245,18 +3564,19 @@
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B2:F58"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -3271,7 +3591,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="4" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -3280,7 +3600,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="9" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="C4" s="6" t="n">
         <f aca="false">COUNTA(B9:B58)</f>
@@ -3289,7 +3609,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="9" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">COUNTIF(E9:E58,"Yes")</f>
@@ -3298,449 +3618,450 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="5" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="13" t="s">
-        <v>173</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>174</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>176</v>
+      <c r="B9" s="17" t="s">
+        <v>180</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="13" t="s">
-        <v>177</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
+      <c r="B10" s="17" t="s">
+        <v>184</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>151</v>
+      </c>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>180</v>
-      </c>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
+      <c r="B11" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="D12" s="13" t="s">
+      <c r="B12" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="17" t="s">
+        <v>189</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>191</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="17" t="s">
+        <v>193</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>194</v>
+      </c>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="C16" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="13" t="s">
-        <v>186</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>187</v>
-      </c>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="13" t="s">
-        <v>188</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>189</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="F15" s="13" t="s">
+      <c r="D16" s="17" t="s">
+        <v>199</v>
+      </c>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="C17" s="17" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>174</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>193</v>
-      </c>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
+      <c r="D17" s="17" t="s">
+        <v>200</v>
+      </c>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>174</v>
-      </c>
-      <c r="D18" s="13" t="s">
-        <v>195</v>
-      </c>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
+      <c r="B18" s="17" t="s">
+        <v>201</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="13"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="13"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
+      <c r="B33" s="17"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="13"/>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="13"/>
+      <c r="B34" s="17"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="13"/>
-      <c r="C35" s="13"/>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
+      <c r="B35" s="17"/>
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="17"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="13"/>
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="13"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="17"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="13"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
-      <c r="F38" s="13"/>
+      <c r="B38" s="17"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="13"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="13"/>
+      <c r="B39" s="17"/>
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="17"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="13"/>
-      <c r="C40" s="13"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="13"/>
-      <c r="F40" s="13"/>
+      <c r="B40" s="17"/>
+      <c r="C40" s="17"/>
+      <c r="D40" s="17"/>
+      <c r="E40" s="17"/>
+      <c r="F40" s="17"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="13"/>
-      <c r="C41" s="13"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="13"/>
-      <c r="F41" s="13"/>
+      <c r="B41" s="17"/>
+      <c r="C41" s="17"/>
+      <c r="D41" s="17"/>
+      <c r="E41" s="17"/>
+      <c r="F41" s="17"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="13"/>
-      <c r="C42" s="13"/>
-      <c r="D42" s="13"/>
-      <c r="E42" s="13"/>
-      <c r="F42" s="13"/>
+      <c r="B42" s="17"/>
+      <c r="C42" s="17"/>
+      <c r="D42" s="17"/>
+      <c r="E42" s="17"/>
+      <c r="F42" s="17"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="13"/>
-      <c r="C43" s="13"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
-      <c r="F43" s="13"/>
+      <c r="B43" s="17"/>
+      <c r="C43" s="17"/>
+      <c r="D43" s="17"/>
+      <c r="E43" s="17"/>
+      <c r="F43" s="17"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="13"/>
-      <c r="C44" s="13"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="13"/>
-      <c r="F44" s="13"/>
+      <c r="B44" s="17"/>
+      <c r="C44" s="17"/>
+      <c r="D44" s="17"/>
+      <c r="E44" s="17"/>
+      <c r="F44" s="17"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="13"/>
-      <c r="C45" s="13"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="13"/>
-      <c r="F45" s="13"/>
+      <c r="B45" s="17"/>
+      <c r="C45" s="17"/>
+      <c r="D45" s="17"/>
+      <c r="E45" s="17"/>
+      <c r="F45" s="17"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="13"/>
-      <c r="C46" s="13"/>
-      <c r="D46" s="13"/>
-      <c r="E46" s="13"/>
-      <c r="F46" s="13"/>
+      <c r="B46" s="17"/>
+      <c r="C46" s="17"/>
+      <c r="D46" s="17"/>
+      <c r="E46" s="17"/>
+      <c r="F46" s="17"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="13"/>
-      <c r="C47" s="13"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="13"/>
-      <c r="F47" s="13"/>
+      <c r="B47" s="17"/>
+      <c r="C47" s="17"/>
+      <c r="D47" s="17"/>
+      <c r="E47" s="17"/>
+      <c r="F47" s="17"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="13"/>
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13"/>
-      <c r="F48" s="13"/>
+      <c r="B48" s="17"/>
+      <c r="C48" s="17"/>
+      <c r="D48" s="17"/>
+      <c r="E48" s="17"/>
+      <c r="F48" s="17"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="13"/>
-      <c r="C49" s="13"/>
-      <c r="D49" s="13"/>
-      <c r="E49" s="13"/>
-      <c r="F49" s="13"/>
+      <c r="B49" s="17"/>
+      <c r="C49" s="17"/>
+      <c r="D49" s="17"/>
+      <c r="E49" s="17"/>
+      <c r="F49" s="17"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="13"/>
-      <c r="C50" s="13"/>
-      <c r="D50" s="13"/>
-      <c r="E50" s="13"/>
-      <c r="F50" s="13"/>
+      <c r="B50" s="17"/>
+      <c r="C50" s="17"/>
+      <c r="D50" s="17"/>
+      <c r="E50" s="17"/>
+      <c r="F50" s="17"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="13"/>
-      <c r="C51" s="13"/>
-      <c r="D51" s="13"/>
-      <c r="E51" s="13"/>
-      <c r="F51" s="13"/>
+      <c r="B51" s="17"/>
+      <c r="C51" s="17"/>
+      <c r="D51" s="17"/>
+      <c r="E51" s="17"/>
+      <c r="F51" s="17"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="13"/>
-      <c r="C52" s="13"/>
-      <c r="D52" s="13"/>
-      <c r="E52" s="13"/>
-      <c r="F52" s="13"/>
+      <c r="B52" s="17"/>
+      <c r="C52" s="17"/>
+      <c r="D52" s="17"/>
+      <c r="E52" s="17"/>
+      <c r="F52" s="17"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="13"/>
-      <c r="C53" s="13"/>
-      <c r="D53" s="13"/>
-      <c r="E53" s="13"/>
-      <c r="F53" s="13"/>
+      <c r="B53" s="17"/>
+      <c r="C53" s="17"/>
+      <c r="D53" s="17"/>
+      <c r="E53" s="17"/>
+      <c r="F53" s="17"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="13"/>
-      <c r="C54" s="13"/>
-      <c r="D54" s="13"/>
-      <c r="E54" s="13"/>
-      <c r="F54" s="13"/>
+      <c r="B54" s="17"/>
+      <c r="C54" s="17"/>
+      <c r="D54" s="17"/>
+      <c r="E54" s="17"/>
+      <c r="F54" s="17"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="13"/>
-      <c r="C55" s="13"/>
-      <c r="D55" s="13"/>
-      <c r="E55" s="13"/>
-      <c r="F55" s="13"/>
+      <c r="B55" s="17"/>
+      <c r="C55" s="17"/>
+      <c r="D55" s="17"/>
+      <c r="E55" s="17"/>
+      <c r="F55" s="17"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="13"/>
-      <c r="C56" s="13"/>
-      <c r="D56" s="13"/>
-      <c r="E56" s="13"/>
-      <c r="F56" s="13"/>
+      <c r="B56" s="17"/>
+      <c r="C56" s="17"/>
+      <c r="D56" s="17"/>
+      <c r="E56" s="17"/>
+      <c r="F56" s="17"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="13"/>
-      <c r="C57" s="13"/>
-      <c r="D57" s="13"/>
-      <c r="E57" s="13"/>
-      <c r="F57" s="13"/>
+      <c r="B57" s="17"/>
+      <c r="C57" s="17"/>
+      <c r="D57" s="17"/>
+      <c r="E57" s="17"/>
+      <c r="F57" s="17"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="13"/>
-      <c r="C58" s="13"/>
-      <c r="D58" s="13"/>
-      <c r="E58" s="13"/>
-      <c r="F58" s="13"/>
+      <c r="B58" s="17"/>
+      <c r="C58" s="17"/>
+      <c r="D58" s="17"/>
+      <c r="E58" s="17"/>
+      <c r="F58" s="17"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="true"/>
   <mergeCells count="1">
     <mergeCell ref="B2:F2"/>
   </mergeCells>
@@ -3749,9 +4070,19 @@
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" error="Pick Yes or No — the use-first counter counts Yes." errorStyle="stop" errorTitle="Pick from the dropdown" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E9:E58" type="list">
+      <formula1>"Yes,No"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C9:C58" type="list">
+      <formula1>"Pantry,Fridge,Freezer,Counter,Garage"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>